<commit_message>
Costing model retuned to 70:30 offshore/onshore with a UAE rate card
CostingModel-DeltaProgramme.xlsx now carries both rate cards and a per-role
onshore share (PM and domain SME fully onshore, architect 60%, leads 40%,
build roles offshore-weighted) landing at exactly 30.0% onshore of the 218
person-months. V15 §16.6/16.7 updated in lockstep: offshore 990,740 +
onshore 1,180,550 = base 2,171,290 (blended ~9,960/MM), 12% contingency
260,555, indicative total 2,431,845 USD.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rfp-response/CostingModel-DeltaProgramme.xlsx
+++ b/rfp-response/CostingModel-DeltaProgramme.xlsx
@@ -68,15 +68,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,12 +443,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,10 +460,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Monthly rate (USD)</t>
+          <t>Offshore rate (USD/mo)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Onshore UAE rate (USD/mo)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -476,9 +483,12 @@
       <c r="B2" s="2" t="n">
         <v>9500</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Programme leadership, governance cadence</t>
+      <c r="C2" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Client-facing governance — onshore-led</t>
         </is>
       </c>
     </row>
@@ -491,9 +501,12 @@
       <c r="B3" s="2" t="n">
         <v>11000</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>AI-native architecture, microservice target</t>
+      <c r="C3" s="2" t="n">
+        <v>24000</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Architecture authority; onshore for design windows</t>
         </is>
       </c>
     </row>
@@ -506,9 +519,12 @@
       <c r="B4" s="2" t="n">
         <v>8000</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>One per major workstream</t>
+      <c r="C4" s="2" t="n">
+        <v>17500</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Workstream leads; onshore rotations</t>
         </is>
       </c>
     </row>
@@ -521,7 +537,10 @@
       <c r="B5" s="2" t="n">
         <v>6500</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Platform and domain services</t>
         </is>
@@ -536,9 +555,12 @@
       <c r="B6" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Feature build, LCNC content</t>
+      <c r="C6" s="2" t="n">
+        <v>11000</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Feature build — offshore</t>
         </is>
       </c>
     </row>
@@ -551,9 +573,12 @@
       <c r="B7" s="2" t="n">
         <v>8500</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Agents, models, evaluation</t>
+      <c r="C7" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Agents, models, evaluation; onshore for AI workshops</t>
         </is>
       </c>
     </row>
@@ -566,9 +591,12 @@
       <c r="B8" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Automation-first testing</t>
+      <c r="C8" s="2" t="n">
+        <v>9500</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Automation-first; onshore for UAT support</t>
         </is>
       </c>
     </row>
@@ -581,7 +609,10 @@
       <c r="B9" s="2" t="n">
         <v>6500</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Chassis, CI/CD, environments</t>
         </is>
@@ -596,9 +627,12 @@
       <c r="B10" s="2" t="n">
         <v>5500</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Maritime domain, UAT support</t>
+      <c r="C10" s="2" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ministry workshops, UAT — onshore-led</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1074,22 +1108,37 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Months each →</t>
+          <t>Person-months</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Person-months</t>
+          <t>Onshore share</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Rate (USD/mo)</t>
+          <t>Onshore MM</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Cost (USD)</t>
+          <t>Offshore MM</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Onshore cost (USD)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Offshore cost (USD)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Role cost (USD)</t>
         </is>
       </c>
     </row>
@@ -1117,17 +1166,31 @@
       <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" s="2">
+      <c r="H2" s="3">
         <f>B2*3+C2*3+D2*3+E2*3+F2*3+G2*1</f>
         <v/>
       </c>
-      <c r="J2" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A2,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K2" s="2">
-        <f>I2*J2</f>
+      <c r="I2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="3">
+        <f>H2*I2</f>
+        <v/>
+      </c>
+      <c r="K2" s="3">
+        <f>H2*(1-I2)</f>
+        <v/>
+      </c>
+      <c r="L2" s="2">
+        <f>J2*INDEX(RateCard!C:C,MATCH(A2,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M2" s="2">
+        <f>K2*INDEX(RateCard!B:B,MATCH(A2,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N2" s="2">
+        <f>L2+M2</f>
         <v/>
       </c>
     </row>
@@ -1155,17 +1218,31 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" s="2">
+      <c r="H3" s="3">
         <f>B3*3+C3*3+D3*3+E3*3+F3*3+G3*1</f>
         <v/>
       </c>
-      <c r="J3" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A3,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K3" s="2">
-        <f>I3*J3</f>
+      <c r="I3" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J3" s="3">
+        <f>H3*I3</f>
+        <v/>
+      </c>
+      <c r="K3" s="3">
+        <f>H3*(1-I3)</f>
+        <v/>
+      </c>
+      <c r="L3" s="2">
+        <f>J3*INDEX(RateCard!C:C,MATCH(A3,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M3" s="2">
+        <f>K3*INDEX(RateCard!B:B,MATCH(A3,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N3" s="2">
+        <f>L3+M3</f>
         <v/>
       </c>
     </row>
@@ -1193,17 +1270,31 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" s="2">
+      <c r="H4" s="3">
         <f>B4*3+C4*3+D4*3+E4*3+F4*3+G4*1</f>
         <v/>
       </c>
-      <c r="J4" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A4,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K4" s="2">
-        <f>I4*J4</f>
+      <c r="I4" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J4" s="3">
+        <f>H4*I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="3">
+        <f>H4*(1-I4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="2">
+        <f>J4*INDEX(RateCard!C:C,MATCH(A4,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M4" s="2">
+        <f>K4*INDEX(RateCard!B:B,MATCH(A4,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N4" s="2">
+        <f>L4+M4</f>
         <v/>
       </c>
     </row>
@@ -1231,17 +1322,31 @@
       <c r="G5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" s="2">
+      <c r="H5" s="3">
         <f>B5*3+C5*3+D5*3+E5*3+F5*3+G5*1</f>
         <v/>
       </c>
-      <c r="J5" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A5,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K5" s="2">
-        <f>I5*J5</f>
+      <c r="I5" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J5" s="3">
+        <f>H5*I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="3">
+        <f>H5*(1-I5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="2">
+        <f>J5*INDEX(RateCard!C:C,MATCH(A5,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M5" s="2">
+        <f>K5*INDEX(RateCard!B:B,MATCH(A5,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N5" s="2">
+        <f>L5+M5</f>
         <v/>
       </c>
     </row>
@@ -1269,17 +1374,31 @@
       <c r="G6" t="n">
         <v>1</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" s="2">
+      <c r="H6" s="3">
         <f>B6*3+C6*3+D6*3+E6*3+F6*3+G6*1</f>
         <v/>
       </c>
-      <c r="J6" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A6,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K6" s="2">
-        <f>I6*J6</f>
+      <c r="I6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3">
+        <f>H6*I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="3">
+        <f>H6*(1-I6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="2">
+        <f>J6*INDEX(RateCard!C:C,MATCH(A6,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M6" s="2">
+        <f>K6*INDEX(RateCard!B:B,MATCH(A6,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N6" s="2">
+        <f>L6+M6</f>
         <v/>
       </c>
     </row>
@@ -1307,17 +1426,31 @@
       <c r="G7" t="n">
         <v>0.5</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" s="2">
+      <c r="H7" s="3">
         <f>B7*3+C7*3+D7*3+E7*3+F7*3+G7*1</f>
         <v/>
       </c>
-      <c r="J7" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A7,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K7" s="2">
-        <f>I7*J7</f>
+      <c r="I7" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J7" s="3">
+        <f>H7*I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="3">
+        <f>H7*(1-I7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="2">
+        <f>J7*INDEX(RateCard!C:C,MATCH(A7,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M7" s="2">
+        <f>K7*INDEX(RateCard!B:B,MATCH(A7,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N7" s="2">
+        <f>L7+M7</f>
         <v/>
       </c>
     </row>
@@ -1345,17 +1478,31 @@
       <c r="G8" t="n">
         <v>1.5</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" s="2">
+      <c r="H8" s="3">
         <f>B8*3+C8*3+D8*3+E8*3+F8*3+G8*1</f>
         <v/>
       </c>
-      <c r="J8" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A8,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K8" s="2">
-        <f>I8*J8</f>
+      <c r="I8" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J8" s="3">
+        <f>H8*I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="3">
+        <f>H8*(1-I8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="2">
+        <f>J8*INDEX(RateCard!C:C,MATCH(A8,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M8" s="2">
+        <f>K8*INDEX(RateCard!B:B,MATCH(A8,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N8" s="2">
+        <f>L8+M8</f>
         <v/>
       </c>
     </row>
@@ -1383,17 +1530,31 @@
       <c r="G9" t="n">
         <v>0.5</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" s="2">
+      <c r="H9" s="3">
         <f>B9*3+C9*3+D9*3+E9*3+F9*3+G9*1</f>
         <v/>
       </c>
-      <c r="J9" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A9,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K9" s="2">
-        <f>I9*J9</f>
+      <c r="I9" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J9" s="3">
+        <f>H9*I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="3">
+        <f>H9*(1-I9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="2">
+        <f>J9*INDEX(RateCard!C:C,MATCH(A9,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M9" s="2">
+        <f>K9*INDEX(RateCard!B:B,MATCH(A9,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N9" s="2">
+        <f>L9+M9</f>
         <v/>
       </c>
     </row>
@@ -1421,24 +1582,38 @@
       <c r="G10" t="n">
         <v>0.5</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" s="2">
+      <c r="H10" s="3">
         <f>B10*3+C10*3+D10*3+E10*3+F10*3+G10*1</f>
         <v/>
       </c>
-      <c r="J10" s="2">
-        <f>INDEX(RateCard!B:B,MATCH(A10,RateCard!A:A,0))</f>
-        <v/>
-      </c>
-      <c r="K10" s="2">
-        <f>I10*J10</f>
+      <c r="I10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="3">
+        <f>H10*I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="3">
+        <f>H10*(1-I10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="2">
+        <f>J10*INDEX(RateCard!C:C,MATCH(A10,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="M10" s="2">
+        <f>K10*INDEX(RateCard!B:B,MATCH(A10,RateCard!A:A,0))</f>
+        <v/>
+      </c>
+      <c r="N10" s="2">
+        <f>L10+M10</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Total FTE / window</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B11" s="4">
@@ -1465,15 +1640,53 @@
         <f>SUM(G2:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="6">
-        <f>SUM(I2:I10)</f>
-        <v/>
-      </c>
-      <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="6">
+      <c r="H11" s="5">
+        <f>SUM(H2:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="5">
+        <f>SUM(J2:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="5">
         <f>SUM(K2:K10)</f>
         <v/>
+      </c>
+      <c r="L11" s="8">
+        <f>SUM(L2:L10)</f>
+        <v/>
+      </c>
+      <c r="M11" s="8">
+        <f>SUM(M2:M10)</f>
+        <v/>
+      </c>
+      <c r="N11" s="8">
+        <f>SUM(N2:N10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Split check</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" s="6">
+        <f>J11/H11</f>
+        <v/>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>(onshore share of MM — target 30%)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1487,11 +1700,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1515,43 +1728,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Programme effort cost</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TeamPlan role mix × RateCard</t>
-        </is>
+          <t>Offshore effort cost</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>ROUND(TeamPlan!K11,1)&amp;" MM at the offshore rate card"</f>
+        <v/>
       </c>
       <c r="C2" s="2">
-        <f>TeamPlan!K11</f>
+        <f>TeamPlan!M11</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Rate below on effort cost</t>
-        </is>
+          <t>Onshore (UAE) effort cost</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>ROUND(TeamPlan!J11,1)&amp;" MM at the UAE rate card"</f>
+        <v/>
       </c>
       <c r="C3" s="2">
-        <f>C2*B5</f>
+        <f>TeamPlan!L11</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Indicative programme total</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="6">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Programme effort cost</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>70:30 offshore/onshore</t>
+        </is>
+      </c>
+      <c r="C4" s="2">
         <f>C2+C3</f>
         <v/>
       </c>
@@ -1559,74 +1774,118 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Contingency rate</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>editable</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0.12</v>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rate below on effort cost</t>
+        </is>
+      </c>
+      <c r="C5" s="2">
+        <f>C4*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Indicative programme total</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="8">
+        <f>C4+C5</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Blended rate check</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>USD per person-month</t>
-        </is>
-      </c>
-      <c r="C7">
-        <f>C2/TeamPlan!I11</f>
-        <v/>
+          <t>Contingency rate</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>editable</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Excluded — passed through at cost:</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>Blended rate check</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>USD per person-month</t>
+        </is>
+      </c>
+      <c r="C9" s="2">
+        <f>C4/TeamPlan!H11</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · Azure consumption and licences</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · AI model usage</t>
-        </is>
+          <t>Onshore share check</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>of person-months</t>
+        </is>
+      </c>
+      <c r="C10" s="6">
+        <f>TeamPlan!J11/TeamPlan!H11</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · Penetration-testing vendors</t>
-        </is>
-      </c>
+          <t>Excluded — passed through at cost:</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · UAE PASS / ICP / payment-gateway / data-provider onboarding fees</t>
+          <t xml:space="preserve">  · Azure consumption and licences</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · Travel</t>
+          <t xml:space="preserve">  · AI model usage</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · Penetration-testing vendors</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · UAE PASS / ICP / payment-gateway / data-provider onboarding fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · International travel (onshore rates are inclusive of local UAE costs)</t>
         </is>
       </c>
     </row>

</xml_diff>